<commit_message>
docs: hoan thien bo tai lieu khoi dong chuan mau Google Sheet va scripts tu dong hoa
</commit_message>
<xml_diff>
--- a/khởi động/CineMax_AI_KhaoSatChucNang_Database_ChiTiet.xlsx
+++ b/khởi động/CineMax_AI_KhaoSatChucNang_Database_ChiTiet.xlsx
@@ -7,11 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Thong_Tin_Du_An" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Khao_Sat_Chuc_Nang_WBS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Thiet_Ke_CSDL_Chi_Tiet" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Quy_Trinh_Nghiep_Vu" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Thong_Tin_Du_An" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Khao_Sat_Chuc_Nang_WBS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Thiet_Ke_CSDL_Chi_Tiet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Quy_Trinh_Nghiep_Vu" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -630,20 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="B2:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -655,7 +641,6 @@
     <col width="21" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -677,7 +662,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -835,8 +819,6 @@
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="8" t="n"/>
     </row>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
@@ -1013,13 +995,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="B2:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1033,7 +1015,6 @@
     <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1048,7 +1029,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="9" t="inlineStr">
         <is>
@@ -2272,13 +2252,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="B2:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2292,7 +2272,6 @@
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2307,7 +2286,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="9" t="inlineStr">
         <is>
@@ -2356,13 +2334,13 @@
           <t>BẢNG DỮ LIỆU: USERS</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="17" t="inlineStr">
@@ -2736,20 +2714,19 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: CINEMAS</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="n"/>
-      <c r="H18" s="20" t="n"/>
-      <c r="I18" s="20" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="17" t="inlineStr">
@@ -2979,20 +2956,19 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="B26" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: ROOMS</t>
         </is>
       </c>
-      <c r="C26" s="20" t="n"/>
-      <c r="D26" s="20" t="n"/>
-      <c r="E26" s="20" t="n"/>
-      <c r="F26" s="20" t="n"/>
-      <c r="G26" s="20" t="n"/>
-      <c r="H26" s="20" t="n"/>
-      <c r="I26" s="20" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="17" t="inlineStr">
@@ -3226,20 +3202,19 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="B34" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: MOVIES</t>
         </is>
       </c>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="20" t="n"/>
-      <c r="F34" s="20" t="n"/>
-      <c r="G34" s="20" t="n"/>
-      <c r="H34" s="20" t="n"/>
-      <c r="I34" s="20" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
+      <c r="I34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="17" t="inlineStr">
@@ -3689,20 +3664,19 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="B48" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: SHOWTIMES</t>
         </is>
       </c>
-      <c r="C48" s="20" t="n"/>
-      <c r="D48" s="20" t="n"/>
-      <c r="E48" s="20" t="n"/>
-      <c r="F48" s="20" t="n"/>
-      <c r="G48" s="20" t="n"/>
-      <c r="H48" s="20" t="n"/>
-      <c r="I48" s="20" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="B49" s="17" t="inlineStr">
@@ -4080,20 +4054,19 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="B60" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: SEAT_LAYOUTS</t>
         </is>
       </c>
-      <c r="C60" s="20" t="n"/>
-      <c r="D60" s="20" t="n"/>
-      <c r="E60" s="20" t="n"/>
-      <c r="F60" s="20" t="n"/>
-      <c r="G60" s="20" t="n"/>
-      <c r="H60" s="20" t="n"/>
-      <c r="I60" s="20" t="n"/>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="7" t="n"/>
+      <c r="E60" s="7" t="n"/>
+      <c r="F60" s="7" t="n"/>
+      <c r="G60" s="7" t="n"/>
+      <c r="H60" s="7" t="n"/>
+      <c r="I60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="B61" s="17" t="inlineStr">
@@ -4281,20 +4254,19 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="B67" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: SEAT_HOLDS</t>
         </is>
       </c>
-      <c r="C67" s="20" t="n"/>
-      <c r="D67" s="20" t="n"/>
-      <c r="E67" s="20" t="n"/>
-      <c r="F67" s="20" t="n"/>
-      <c r="G67" s="20" t="n"/>
-      <c r="H67" s="20" t="n"/>
-      <c r="I67" s="20" t="n"/>
+      <c r="C67" s="7" t="n"/>
+      <c r="D67" s="7" t="n"/>
+      <c r="E67" s="7" t="n"/>
+      <c r="F67" s="7" t="n"/>
+      <c r="G67" s="7" t="n"/>
+      <c r="H67" s="7" t="n"/>
+      <c r="I67" s="8" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="13" t="inlineStr">
@@ -4520,20 +4492,19 @@
         </is>
       </c>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="B75" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: BOOKINGS</t>
         </is>
       </c>
-      <c r="C75" s="20" t="n"/>
-      <c r="D75" s="20" t="n"/>
-      <c r="E75" s="20" t="n"/>
-      <c r="F75" s="20" t="n"/>
-      <c r="G75" s="20" t="n"/>
-      <c r="H75" s="20" t="n"/>
-      <c r="I75" s="20" t="n"/>
+      <c r="C75" s="7" t="n"/>
+      <c r="D75" s="7" t="n"/>
+      <c r="E75" s="7" t="n"/>
+      <c r="F75" s="7" t="n"/>
+      <c r="G75" s="7" t="n"/>
+      <c r="H75" s="7" t="n"/>
+      <c r="I75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="13" t="inlineStr">
@@ -5055,20 +5026,19 @@
         </is>
       </c>
     </row>
-    <row r="90"/>
     <row r="91">
       <c r="B91" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: TICKETS</t>
         </is>
       </c>
-      <c r="C91" s="20" t="n"/>
-      <c r="D91" s="20" t="n"/>
-      <c r="E91" s="20" t="n"/>
-      <c r="F91" s="20" t="n"/>
-      <c r="G91" s="20" t="n"/>
-      <c r="H91" s="20" t="n"/>
-      <c r="I91" s="20" t="n"/>
+      <c r="C91" s="7" t="n"/>
+      <c r="D91" s="7" t="n"/>
+      <c r="E91" s="7" t="n"/>
+      <c r="F91" s="7" t="n"/>
+      <c r="G91" s="7" t="n"/>
+      <c r="H91" s="7" t="n"/>
+      <c r="I91" s="8" t="n"/>
     </row>
     <row r="92">
       <c r="B92" s="13" t="inlineStr">
@@ -5332,20 +5302,19 @@
         </is>
       </c>
     </row>
-    <row r="99"/>
     <row r="100">
       <c r="B100" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: VOUCHERS</t>
         </is>
       </c>
-      <c r="C100" s="20" t="n"/>
-      <c r="D100" s="20" t="n"/>
-      <c r="E100" s="20" t="n"/>
-      <c r="F100" s="20" t="n"/>
-      <c r="G100" s="20" t="n"/>
-      <c r="H100" s="20" t="n"/>
-      <c r="I100" s="20" t="n"/>
+      <c r="C100" s="7" t="n"/>
+      <c r="D100" s="7" t="n"/>
+      <c r="E100" s="7" t="n"/>
+      <c r="F100" s="7" t="n"/>
+      <c r="G100" s="7" t="n"/>
+      <c r="H100" s="7" t="n"/>
+      <c r="I100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="B101" s="17" t="inlineStr">
@@ -5741,20 +5710,19 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="B113" s="19" t="inlineStr">
         <is>
           <t>BẢNG DỮ LIỆU: REVIEWS</t>
         </is>
       </c>
-      <c r="C113" s="20" t="n"/>
-      <c r="D113" s="20" t="n"/>
-      <c r="E113" s="20" t="n"/>
-      <c r="F113" s="20" t="n"/>
-      <c r="G113" s="20" t="n"/>
-      <c r="H113" s="20" t="n"/>
-      <c r="I113" s="20" t="n"/>
+      <c r="C113" s="7" t="n"/>
+      <c r="D113" s="7" t="n"/>
+      <c r="E113" s="7" t="n"/>
+      <c r="F113" s="7" t="n"/>
+      <c r="G113" s="7" t="n"/>
+      <c r="H113" s="7" t="n"/>
+      <c r="I113" s="8" t="n"/>
     </row>
     <row r="114">
       <c r="B114" s="13" t="inlineStr">
@@ -6064,8 +6032,8 @@
   <mergeCells count="11">
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B100:I100"/>
     <mergeCell ref="B75:I75"/>
-    <mergeCell ref="B100:I100"/>
     <mergeCell ref="B91:I91"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B34:I34"/>
@@ -6078,13 +6046,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="B2:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6096,7 +6064,6 @@
     <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -6111,7 +6078,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="9" t="inlineStr">
         <is>
@@ -6150,11 +6116,11 @@
           <t>Quy Trình 1: Đặt Vé &amp; Giữ Ghế Nguyên Tử 300s (Seat Hold &amp; Booking)</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="14" t="inlineStr">
@@ -6316,18 +6282,17 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Quy Trình 2: Soát Vé Điện Tử Tại Cửa Bằng Mã QR (Anti-Fraud Scanner)</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="10" t="inlineStr">
@@ -6489,18 +6454,17 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Quy Trình 3: Xếp Lịch Chiếu &amp; Kiểm Tra Va Chạm Phòng (Collision Engine)</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n"/>
-      <c r="D20" s="20" t="n"/>
-      <c r="E20" s="20" t="n"/>
-      <c r="F20" s="20" t="n"/>
-      <c r="G20" s="20" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -6630,18 +6594,17 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="B26" s="19" t="inlineStr">
         <is>
           <t>Quy Trình 4: Quy Trình Xử Lý Hoàn Trả &amp; Hủy Vé 6 Bước (Refund Policy)</t>
         </is>
       </c>
-      <c r="C26" s="20" t="n"/>
-      <c r="D26" s="20" t="n"/>
-      <c r="E26" s="20" t="n"/>
-      <c r="F26" s="20" t="n"/>
-      <c r="G26" s="20" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="14" t="inlineStr">

</xml_diff>